<commit_message>
another version with other type of aligmnet and branches creator for what suppos to be now more accurate istoype based tree, also with more accurate mutations per branch and new visualizations for the tree and the mutations per branch, also with a new function to create a table with the mutations per branch and the isotypes of each branch, this table is in the results folder as mutations_per_branch.xlsx
</commit_message>
<xml_diff>
--- a/results/385_1/mutations_per_branch.xlsx
+++ b/results/385_1/mutations_per_branch.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Pythoncourse42026\Final-project-BCR-Lineage-Tracer\results\385_1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE79949B-5DB6-46E6-9A93-4234670F4BBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CD1200D-DDA9-4AF1-9E49-7F0609FD7756}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1222,7 +1222,7 @@
       <xdr:col>14</xdr:col>
       <xdr:colOff>228057</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>6456</xdr:rowOff>
+      <xdr:rowOff>9482</xdr:rowOff>
     </xdr:to>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
@@ -1601,71 +1601,6 @@
     </mc:AlternateContent>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>23</xdr:col>
-      <xdr:colOff>7582</xdr:colOff>
-      <xdr:row>33</xdr:row>
-      <xdr:rowOff>23510</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>23</xdr:col>
-      <xdr:colOff>154462</xdr:colOff>
-      <xdr:row>34</xdr:row>
-      <xdr:rowOff>18788</xdr:rowOff>
-    </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
-        <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId34">
-          <xdr14:nvContentPartPr>
-            <xdr14:cNvPr id="43" name="דיו 42">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A3B019A5-994F-35DC-997C-C1D8C86F2453}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr14:cNvPr>
-            <xdr14:cNvContentPartPr/>
-          </xdr14:nvContentPartPr>
-          <xdr14:nvPr macro=""/>
-          <xdr14:xfrm>
-            <a:off x="18652770" y="6048073"/>
-            <a:ext cx="146880" cy="177840"/>
-          </xdr14:xfrm>
-        </xdr:contentPart>
-      </mc:Choice>
-      <mc:Fallback>
-        <xdr:pic>
-          <xdr:nvPicPr>
-            <xdr:cNvPr id="43" name="דיו 42">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A3B019A5-994F-35DC-997C-C1D8C86F2453}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvPicPr/>
-          </xdr:nvPicPr>
-          <xdr:blipFill>
-            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId35"/>
-            <a:stretch>
-              <a:fillRect/>
-            </a:stretch>
-          </xdr:blipFill>
-          <xdr:spPr>
-            <a:xfrm>
-              <a:off x="18617130" y="6012433"/>
-              <a:ext cx="218520" cy="249480"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-          </xdr:spPr>
-        </xdr:pic>
-      </mc:Fallback>
-    </mc:AlternateContent>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -1898,34 +1833,6 @@
     </inkml:brush>
   </inkml:definitions>
   <inkml:trace contextRef="#ctx0" brushRef="#br0">0 1,'3'0,"5"0,3 0,4 0,2 0,1 0,2 0,-1 0,1 0,-4 0</inkml:trace>
-</inkml:ink>
-</file>
-
-<file path=xl/ink/ink17.xml><?xml version="1.0" encoding="utf-8"?>
-<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
-  <inkml:definitions>
-    <inkml:context xml:id="ctx0">
-      <inkml:inkSource xml:id="inkSrc0">
-        <inkml:traceFormat>
-          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
-        </inkml:traceFormat>
-        <inkml:channelProperties>
-          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
-        </inkml:channelProperties>
-      </inkml:inkSource>
-      <inkml:timestamp xml:id="ts0" timeString="2026-06-03T12:59:25.760"/>
-    </inkml:context>
-    <inkml:brush xml:id="br0">
-      <inkml:brushProperty name="width" value="0.2" units="cm"/>
-      <inkml:brushProperty name="height" value="0.2" units="cm"/>
-      <inkml:brushProperty name="color" value="#849398"/>
-    </inkml:brush>
-  </inkml:definitions>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0">4498 3151 24575,'2'34'0,"9"54"0,-1-21 0,-4-34 0,1 0 0,2 0 0,26 60 0,-12-32 0,-21-58 0,-1 0 0,1 0 0,0 0 0,0 0 0,0 0 0,1 0 0,-1-1 0,1 1 0,-1-1 0,1 1 0,0-1 0,0 0 0,0 0 0,0-1 0,0 1 0,0 0 0,1-1 0,-1 0 0,1 0 0,-1 0 0,1 0 0,-1 0 0,1-1 0,3 0 0,15 2 0,-1-2 0,1 0 0,22-4 0,-1 1 0,35 2-1365</inkml:trace>
 </inkml:ink>
 </file>
 

</xml_diff>